<commit_message>
feat: add Excel template for LMS question imports
</commit_message>
<xml_diff>
--- a/outputs/question-import-template/Template_Import_Soal_LMS.xlsx
+++ b/outputs/question-import-template/Template_Import_Soal_LMS.xlsx
@@ -301,7 +301,7 @@
     <t>generated_at</t>
   </si>
   <si>
-    <t>2026-08-29T14:24:31.032Z</t>
+    <t>2026-08-29T14:35:50.972Z</t>
   </si>
   <si>
     <t>Tipe Soal</t>
@@ -1108,7 +1108,7 @@
       <c r="C20" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="QHjk7mGzO8Aq8jWTvtNySTkqsovgefb35Wseal3j2pNIsIEW/lSufJdWJWdOEbtf7NZRWcsbbDYmbvEnMe3Ebg==" saltValue="SU6NeJensl37vx/iU4xfBw==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="iyezppL464tTCye49c0mDTHA5ERWFI6R0sDd42KbbC2d8+BK5VhI0hqT55ABWgnfcplNDPkhg2XtsjfPrcNzCw==" saltValue="X27Jl8V6Lw/Xnk7/DqAwxg==" spinCount="100000"/>
   <mergeCells count="8">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -33542,7 +33542,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="RNdLAzYepslpIuyMtuzyhF8qhVhIdiFXTCle8DOWTykNhLCp4kiIBgQAGRNwmsU4giqxTFGXoU5oenOqK4t1fQ==" saltValue="IMK9xkRPumdS/FGzVOMG3Q==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="EvaarMI3SUyUwd6W7RuV4dVkdSCfB1y8nTmodJsq5sPFjcFFu445wpPbIX0fZYz31SOS0ffPhstEkOGbrmg6TA==" saltValue="RnaJ6OkCmSXJqzKMoHaHtg==" spinCount="100000"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -33613,7 +33613,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="rKVRadb2p//t5G2702i181YKJmkxJV18iio66KpWpGvpsqwMDSP1k4rsmnkW8R7Sqm5ZezagyJ5wjh+GI5AE1A==" saltValue="odfv32HJeUf75eFu9snkrQ==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="c7v44Ok/qBcVfPqJp0pcrTJZNWe7zAyHMqa4H8nTz02qBJ9NMdW5IKO7VD6LzUHChtJk7Obr1plHFcRmUAOS1Q==" saltValue="MN1jDunmVqa1ueIUrxymYg==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -33740,7 +33740,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="DAP6ngWIO5I4zx5oIf2GFfCXdKnibincSzLElDqFWi263eQtNwwmagqYSzVPhg1A8Cb9uQv5UdnS6JmHB67QEg==" saltValue="++sFP5/yULUz74t/1+un7A==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="HNIlJXA0a7Ngqo6Pzef/wvxW7KXSnL3XZfu+wxodbUWHRPRynHEGlspRTAWHFF46qWYul0mWzrpiyq65lcnFMA==" saltValue="VFGLjfIU209LwIqxWeC5iw==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>